<commit_message>
bash & ssh & JVMTI & 装修
</commit_message>
<xml_diff>
--- a/life/house/家居_装修/2018_临江花园装修记录/临江花园预算清单.xlsx
+++ b/life/house/家居_装修/2018_临江花园装修记录/临江花园预算清单.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="28125"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="28600" yWindow="20740" windowWidth="25600" windowHeight="16680" tabRatio="500"/>
+    <workbookView xWindow="240" yWindow="240" windowWidth="25360" windowHeight="15820" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="380">
   <si>
     <t>中亚海外购</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -1021,309 +1021,490 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>净水器单独计算</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>总费用</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>卫浴设备总费用</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>台盆、马桶、浴缸</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>台盆</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>杜拉维特</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>杜拉维特</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>马桶</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>科勒</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>浴缸</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>门窗</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>凤铝</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>次卧</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>铝合金窗</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>卧室门</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>入室门</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>门窗总费用</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>无类别小项总费用</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>厨卫电器总费用</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>电器总费用</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>电器</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>冰箱</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>洗衣机</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>烘衣机</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>暖通总费用</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>暖通量大，而且是系统工程，所以单独从电器拿出来</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>总价</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>级别</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>状态</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>备注</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>空调</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>地暖</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>新风</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>家具总费用</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>成品家具总费用</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>定制家具总费用</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>木工家具总费用</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>厨卫五金总花费</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GROHE Bau Cosmopolitan | Badaccessoires - Handtuch | Bademantelhaken | 40461001</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>高仪·浴室·挂钩·40461001</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>浴室五金·挂钩</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>五金</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>卫生间</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GROHE Original WAS | Sicherungstechnik - Kombi-Eckventil | mit selbstdichtendem Anschlussgewinde, Wandanschluss 1/2 Zoll, Abgang 3/8 Zoll, Abgang 3/4</t>
+  </si>
+  <si>
+    <t>德亚</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>洗衣机龙头带角阀功能</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>高仪洗衣机龙头带角阀功能</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GROHE Essentials | Badaccessoires - Seifenspender | mit Halter | 40448001</t>
+  </si>
+  <si>
+    <t>浴室五金·洗手液瓶</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>高仪·浴室·洗手液瓶·40448001</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>浴室五金·卫生纸托</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GROHE Essentials | Badaccessoires - WC-Papierrollenhalter | mit Deckel, chrom | 40367001</t>
+  </si>
+  <si>
+    <t>高仪·浴室·卫生纸托·40367001</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>浴室五金·单杆衣架</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Grohe Bau Cosmopolitan Badaccessoires - Badetuchhalter, 40459001</t>
+  </si>
+  <si>
+    <t>高仪·浴室·单杆衣架·40459001</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>浴室五金·双杆可转动衣架</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>高仪·浴室·双杆可转动衣架·40371001</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GROHE Essentials | Badaccessoires - Bademantelhaken | chrom | 40364001</t>
+  </si>
+  <si>
+    <t>高仪·浴室·挂钩·40364001</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>浴室五金·大挂钩</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>高仪·浴室·大挂钩·40511001</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Grohe Essentials Halter, Glas Seifenschale, chrom, 40369001</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>浴室五金·洗漱杯托</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>高仪·浴室·洗漱杯托·40369001</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>浴室五金·毛巾环</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>高仪·浴室·毛巾环·40365001</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>浴室五金·浴液托</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>高仪·浴室·浴液托·40659001</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Grohe Essentials Authentic Ablagekorb, klein, chrom, 40659001</t>
+  </si>
+  <si>
+    <t>茶室</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>玻璃移门</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>书房</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>玻璃展示区+玻璃门</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>淋浴房</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>浴缸上方玻璃墙+玻璃门</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>润美</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>70开窗、5-27A-5、全部内开内倒、ROTO、外面烤漆灰色、南面玻璃low-E。 付了2k定金；</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>长度522；离墙55</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>长度439； 高低54</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>环直径180； 高低201； 离墙44； 固定处高低54</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>长度134；；高低46； 固定处高低44</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>无类别大项总费用</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>瓷砖</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>瓷砖</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>亿丰-伊罗丹妮</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>含搬运上楼（电梯）； 已付3000定金；</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>半包总费用</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>半包合同费用</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>半包</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>腻子粉增项</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>半包增项</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>美巢800JJ换GQ，工料总增</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>入户线</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>三相五根10方入户，工料（电线、线管、人工等）总增。 这个有点贵，估计1600就够了，不计较了</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>净水器系统总费用</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>净水器单独计算</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>总费用</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>卫浴设备总费用</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>台盆、马桶、浴缸</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>台盆</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>杜拉维特</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>杜拉维特</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>马桶</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>科勒</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>浴缸</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>门窗</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>润美</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>凤铝</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>次卧</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>铝合金窗</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>卧室门</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>入室门</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>门窗总费用</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>无类别小项总费用</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>厨卫电器总费用</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>电器总费用</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>电器</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>冰箱</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>洗衣机</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>烘衣机</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>暖通总费用</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>暖通量大，而且是系统工程，所以单独从电器拿出来</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>总价</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>级别</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>状态</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>备注</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>空调</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>地暖</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>新风</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>家具总费用</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>成品家具总费用</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>定制家具总费用</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>木工家具总费用</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>厨卫五金总花费</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>GROHE Bau Cosmopolitan | Badaccessoires - Handtuch | Bademantelhaken | 40461001</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>高仪·浴室·挂钩·40461001</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>浴室五金·挂钩</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>五金</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>卫生间</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>GROHE Original WAS | Sicherungstechnik - Kombi-Eckventil | mit selbstdichtendem Anschlussgewinde, Wandanschluss 1/2 Zoll, Abgang 3/8 Zoll, Abgang 3/4</t>
-  </si>
-  <si>
-    <t>德亚</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>洗衣机龙头带角阀功能</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>高仪洗衣机龙头带角阀功能</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>GROHE Essentials | Badaccessoires - Seifenspender | mit Halter | 40448001</t>
-  </si>
-  <si>
-    <t>浴室五金·洗手液瓶</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>高仪·浴室·洗手液瓶·40448001</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>浴室五金·卫生纸托</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>GROHE Essentials | Badaccessoires - WC-Papierrollenhalter | mit Deckel, chrom | 40367001</t>
-  </si>
-  <si>
-    <t>高仪·浴室·卫生纸托·40367001</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>浴室五金·单杆衣架</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Grohe Bau Cosmopolitan Badaccessoires - Badetuchhalter, 40459001</t>
-  </si>
-  <si>
-    <t>高仪·浴室·单杆衣架·40459001</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>浴室五金·双杆可转动衣架</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>高仪·浴室·双杆可转动衣架·40371001</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>GROHE Essentials | Badaccessoires - Bademantelhaken | chrom | 40364001</t>
-  </si>
-  <si>
-    <t>高仪·浴室·挂钩·40364001</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>浴室五金·大挂钩</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>高仪·浴室·大挂钩·40511001</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Grohe Essentials Halter, Glas Seifenschale, chrom, 40369001</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>浴室五金·洗漱杯托</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>高仪·浴室·洗漱杯托·40369001</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>浴室五金·毛巾环</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>高仪·浴室·毛巾环·40365001</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>浴室五金·浴液托</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>高仪·浴室·浴液托·40659001</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Grohe Essentials Authentic Ablagekorb, klein, chrom, 40659001</t>
-  </si>
-  <si>
-    <t>茶室</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>玻璃移门</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>书房</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>玻璃展示区+玻璃门</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>淋浴房</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>浴缸上方玻璃墙+玻璃门</t>
+    <t>水路系统总费用</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>格兰富</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>丹麦格兰富水泵CM5-4PC自动加压泵增压泵家用自来水增压泵稳压泵</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>增压泵</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>CM5-4PC</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>格兰富·CM5-4PC·增压泵</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>淘宝</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>含过滤阀门</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>德亚直邮</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>打包费用</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>APP遥控空调</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>空调彩屏面板</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>管线机</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>科勒·拂乐·1.8m</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>科勒拂乐K-99211T-0/99210/99212嵌入式1.7/1.6/1.8米铸铁浴缸</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>厨房总费用</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>水槽</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>铂浪高</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>水槽</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Blanco 铂浪高 LEXA 8S, 厨房水槽, Silgranit PuraDur花岗岩水槽, 单槽, 沥青色, 514708 </t>
+  </si>
+  <si>
+    <t>铂浪高·LEXA 8S·花岗岩水槽</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>中亚海外购</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>喷枪龙头套餐</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Hansgrohe – Intimate 马桶厕所淋浴 bidette </t>
+  </si>
+  <si>
+    <t>汉斯格雅·intimate·喷枪花洒套装</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Grohe 高仪 Tempesta-F 清洁喷雾器，带支架和角阀，喷射等级 1 级，27514001</t>
+  </si>
+  <si>
+    <t>喷枪</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>高仪·tempesta-F·喷枪</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1331,7 +1512,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1380,6 +1561,15 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="2"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -1422,7 +1612,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="77">
+  <cellStyleXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -1500,8 +1690,41 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1510,8 +1733,9 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="77">
+  <cellStyles count="110">
     <cellStyle name="超链接" xfId="1" builtinId="8"/>
     <cellStyle name="访问过的超链接" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="访问过的超链接" xfId="3" builtinId="9" hidden="1"/>
@@ -1588,6 +1812,39 @@
     <cellStyle name="访问过的超链接" xfId="74" builtinId="9" hidden="1"/>
     <cellStyle name="访问过的超链接" xfId="75" builtinId="9" hidden="1"/>
     <cellStyle name="访问过的超链接" xfId="76" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="77" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="78" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="79" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="80" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="81" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="82" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="83" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="84" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="85" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="86" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="87" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="88" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="89" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="90" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="91" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="92" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="93" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="94" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="95" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="96" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="97" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="98" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="99" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="100" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="101" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="102" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="103" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="104" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="105" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="106" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="107" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="108" builtinId="9" hidden="1"/>
+    <cellStyle name="访问过的超链接" xfId="109" builtinId="9" hidden="1"/>
     <cellStyle name="普通" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1917,7 +2174,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P87"/>
+  <dimension ref="A1:P107"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
   <cols>
     <col min="4" max="4" width="15" customWidth="1"/>
@@ -1959,16 +2216,16 @@
         <v>8</v>
       </c>
       <c r="L1" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="M1" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="N1" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="P1" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -2186,31 +2443,34 @@
     </row>
     <row r="9" spans="1:16">
       <c r="A9" t="s">
-        <v>200</v>
+        <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>201</v>
+        <v>158</v>
       </c>
       <c r="C9" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="D9" t="s">
-        <v>303</v>
+        <v>378</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>301</v>
+        <v>377</v>
       </c>
       <c r="F9" t="s">
-        <v>304</v>
+        <v>379</v>
       </c>
       <c r="G9">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>27514001</v>
       </c>
       <c r="J9">
-        <v>356</v>
+        <v>496</v>
       </c>
       <c r="K9" t="s">
-        <v>302</v>
+        <v>0</v>
       </c>
       <c r="L9" t="s">
         <v>148</v>
@@ -2218,37 +2478,31 @@
     </row>
     <row r="10" spans="1:16">
       <c r="A10" t="s">
-        <v>157</v>
+        <v>200</v>
       </c>
       <c r="B10" t="s">
-        <v>158</v>
+        <v>201</v>
       </c>
       <c r="C10" t="s">
         <v>160</v>
       </c>
       <c r="D10" t="s">
-        <v>161</v>
+        <v>301</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>159</v>
+        <v>299</v>
       </c>
       <c r="F10" t="s">
-        <v>162</v>
+        <v>302</v>
       </c>
       <c r="G10">
-        <v>1</v>
-      </c>
-      <c r="H10">
-        <v>13285</v>
-      </c>
-      <c r="I10" t="s">
-        <v>156</v>
+        <v>2</v>
       </c>
       <c r="J10">
-        <v>581.78</v>
+        <v>356</v>
       </c>
       <c r="K10" t="s">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="L10" t="s">
         <v>148</v>
@@ -2259,28 +2513,31 @@
         <v>157</v>
       </c>
       <c r="B11" t="s">
-        <v>171</v>
+        <v>158</v>
       </c>
       <c r="C11" t="s">
-        <v>191</v>
+        <v>160</v>
       </c>
       <c r="D11" t="s">
-        <v>190</v>
+        <v>161</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>188</v>
+        <v>159</v>
       </c>
       <c r="F11" t="s">
-        <v>189</v>
+        <v>162</v>
       </c>
       <c r="G11">
         <v>1</v>
       </c>
       <c r="H11">
-        <v>15984181</v>
+        <v>13285</v>
+      </c>
+      <c r="I11" t="s">
+        <v>156</v>
       </c>
       <c r="J11">
-        <v>757</v>
+        <v>581.78</v>
       </c>
       <c r="K11" t="s">
         <v>0</v>
@@ -2300,60 +2557,63 @@
         <v>191</v>
       </c>
       <c r="D12" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="F12" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="G12">
         <v>1</v>
       </c>
       <c r="H12">
-        <v>15937001</v>
+        <v>15984181</v>
       </c>
       <c r="J12">
-        <v>1075</v>
+        <v>757</v>
       </c>
       <c r="K12" t="s">
         <v>0</v>
       </c>
       <c r="L12" t="s">
-        <v>195</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13" spans="1:16">
       <c r="A13" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="B13" t="s">
-        <v>201</v>
+        <v>171</v>
       </c>
       <c r="C13" t="s">
         <v>191</v>
       </c>
       <c r="D13" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>206</v>
+        <v>192</v>
       </c>
       <c r="F13" t="s">
-        <v>207</v>
+        <v>194</v>
       </c>
       <c r="G13">
         <v>1</v>
       </c>
+      <c r="H13">
+        <v>15937001</v>
+      </c>
       <c r="J13">
-        <v>180</v>
+        <v>1075</v>
       </c>
       <c r="K13" t="s">
         <v>0</v>
       </c>
       <c r="L13" t="s">
-        <v>148</v>
+        <v>195</v>
       </c>
     </row>
     <row r="14" spans="1:16">
@@ -2367,19 +2627,19 @@
         <v>191</v>
       </c>
       <c r="D14" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="F14" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="G14">
         <v>1</v>
       </c>
       <c r="J14">
-        <v>580</v>
+        <v>180</v>
       </c>
       <c r="K14" t="s">
         <v>0</v>
@@ -2399,19 +2659,19 @@
         <v>191</v>
       </c>
       <c r="D15" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="F15" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="G15">
         <v>1</v>
       </c>
       <c r="J15">
-        <v>610</v>
+        <v>580</v>
       </c>
       <c r="K15" t="s">
         <v>0</v>
@@ -2431,22 +2691,19 @@
         <v>191</v>
       </c>
       <c r="D16" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="F16" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="G16">
         <v>1</v>
       </c>
-      <c r="H16">
-        <v>1800180</v>
-      </c>
       <c r="J16">
-        <v>860</v>
+        <v>610</v>
       </c>
       <c r="K16" t="s">
         <v>0</v>
@@ -2466,22 +2723,22 @@
         <v>191</v>
       </c>
       <c r="D17" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="F17" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="G17">
         <v>1</v>
       </c>
       <c r="H17">
-        <v>31743</v>
+        <v>1800180</v>
       </c>
       <c r="J17">
-        <v>1200</v>
+        <v>860</v>
       </c>
       <c r="K17" t="s">
         <v>0</v>
@@ -2501,19 +2758,22 @@
         <v>191</v>
       </c>
       <c r="D18" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F18" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="G18">
         <v>1</v>
       </c>
+      <c r="H18">
+        <v>31743</v>
+      </c>
       <c r="J18">
-        <v>2669</v>
+        <v>1200</v>
       </c>
       <c r="K18" t="s">
         <v>0</v>
@@ -2527,31 +2787,25 @@
         <v>169</v>
       </c>
       <c r="B19" t="s">
-        <v>171</v>
+        <v>201</v>
       </c>
       <c r="C19" t="s">
-        <v>170</v>
+        <v>191</v>
       </c>
       <c r="D19" t="s">
-        <v>173</v>
+        <v>222</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>187</v>
+        <v>218</v>
       </c>
       <c r="F19" t="s">
-        <v>168</v>
+        <v>223</v>
       </c>
       <c r="G19">
-        <v>2</v>
-      </c>
-      <c r="H19">
-        <v>23200000</v>
-      </c>
-      <c r="I19" t="s">
-        <v>172</v>
+        <v>1</v>
       </c>
       <c r="J19">
-        <v>2071</v>
+        <v>2669</v>
       </c>
       <c r="K19" t="s">
         <v>0</v>
@@ -2562,34 +2816,31 @@
     </row>
     <row r="20" spans="1:16">
       <c r="A20" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="B20" t="s">
-        <v>171</v>
+        <v>158</v>
       </c>
       <c r="C20" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="D20" t="s">
-        <v>174</v>
+        <v>374</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>176</v>
+        <v>375</v>
       </c>
       <c r="F20" t="s">
-        <v>177</v>
+        <v>376</v>
       </c>
       <c r="G20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H20">
-        <v>19967001</v>
-      </c>
-      <c r="I20" t="s">
-        <v>175</v>
+        <v>32126000</v>
       </c>
       <c r="J20">
-        <v>2137</v>
+        <v>1010</v>
       </c>
       <c r="K20" t="s">
         <v>0</v>
@@ -2600,1089 +2851,1469 @@
     </row>
     <row r="21" spans="1:16">
       <c r="A21" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="B21" t="s">
-        <v>201</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>235</v>
-      </c>
-      <c r="E21" s="1"/>
-      <c r="J21" s="6">
-        <f>SUM(J10:J20)</f>
-        <v>12720.779999999999</v>
-      </c>
-      <c r="N21">
+        <v>171</v>
+      </c>
+      <c r="C21" t="s">
+        <v>170</v>
+      </c>
+      <c r="D21" t="s">
+        <v>173</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F21" t="s">
+        <v>168</v>
+      </c>
+      <c r="G21">
         <v>2</v>
+      </c>
+      <c r="H21">
+        <v>23200000</v>
+      </c>
+      <c r="I21" t="s">
+        <v>172</v>
+      </c>
+      <c r="J21">
+        <v>2071</v>
+      </c>
+      <c r="K21" t="s">
+        <v>0</v>
+      </c>
+      <c r="L21" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="22" spans="1:16">
       <c r="A22" t="s">
-        <v>233</v>
+        <v>169</v>
       </c>
       <c r="B22" t="s">
-        <v>201</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="E22" s="1"/>
-      <c r="J22" s="6">
-        <f>SUM(J4:J8)</f>
-        <v>3485.79</v>
-      </c>
-      <c r="N22">
+        <v>171</v>
+      </c>
+      <c r="C22" t="s">
+        <v>170</v>
+      </c>
+      <c r="D22" t="s">
+        <v>174</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="F22" t="s">
+        <v>177</v>
+      </c>
+      <c r="G22">
         <v>2</v>
+      </c>
+      <c r="H22">
+        <v>19967001</v>
+      </c>
+      <c r="I22" t="s">
+        <v>175</v>
+      </c>
+      <c r="J22">
+        <v>2137</v>
+      </c>
+      <c r="K22" t="s">
+        <v>0</v>
+      </c>
+      <c r="L22" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="23" spans="1:16">
       <c r="A23" t="s">
-        <v>232</v>
+        <v>157</v>
       </c>
       <c r="B23" t="s">
         <v>201</v>
       </c>
-      <c r="D23" s="3" t="s">
-        <v>237</v>
-      </c>
+      <c r="D23" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="E23" s="1"/>
       <c r="J23" s="6">
-        <f>SUM(J3:J18)</f>
-        <v>13079.970000000001</v>
-      </c>
-      <c r="L23" t="s">
-        <v>231</v>
+        <f>SUM(J11:J22)</f>
+        <v>13730.779999999999</v>
       </c>
       <c r="N23">
-        <v>1</v>
-      </c>
-      <c r="P23">
-        <f>J23</f>
-        <v>13079.970000000001</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:16">
-      <c r="J24" s="6"/>
+      <c r="A24" t="s">
+        <v>233</v>
+      </c>
+      <c r="B24" t="s">
+        <v>201</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="E24" s="1"/>
+      <c r="J24" s="6">
+        <f>SUM(J4:J11)</f>
+        <v>4919.57</v>
+      </c>
+      <c r="N24">
+        <v>2</v>
+      </c>
     </row>
     <row r="25" spans="1:16">
       <c r="A25" t="s">
-        <v>300</v>
+        <v>232</v>
       </c>
       <c r="B25" t="s">
-        <v>299</v>
-      </c>
-      <c r="C25" t="s">
-        <v>160</v>
-      </c>
-      <c r="D25" t="s">
-        <v>306</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>305</v>
-      </c>
-      <c r="F25" t="s">
-        <v>307</v>
-      </c>
-      <c r="G25">
+        <v>201</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="J25" s="6">
+        <f>SUM(J3:J22)</f>
+        <v>18793.97</v>
+      </c>
+      <c r="L25" t="s">
+        <v>231</v>
+      </c>
+      <c r="N25">
         <v>1</v>
       </c>
-      <c r="H25">
-        <v>40448001</v>
-      </c>
-      <c r="J25" s="6">
-        <v>353</v>
+      <c r="P25">
+        <f>J25</f>
+        <v>18793.97</v>
       </c>
     </row>
     <row r="26" spans="1:16">
-      <c r="A26" t="s">
-        <v>300</v>
-      </c>
-      <c r="B26" t="s">
-        <v>299</v>
-      </c>
-      <c r="C26" t="s">
-        <v>160</v>
-      </c>
-      <c r="D26" t="s">
-        <v>311</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>312</v>
-      </c>
-      <c r="F26" t="s">
-        <v>313</v>
-      </c>
-      <c r="G26">
-        <v>2</v>
-      </c>
-      <c r="H26">
-        <v>40459001</v>
-      </c>
-      <c r="J26" s="6">
-        <v>368</v>
-      </c>
+      <c r="J26" s="6"/>
     </row>
     <row r="27" spans="1:16">
       <c r="A27" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B27" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C27" t="s">
         <v>160</v>
       </c>
       <c r="D27" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="F27" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
       <c r="G27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H27">
-        <v>40371001</v>
+        <v>40448001</v>
       </c>
       <c r="J27" s="6">
-        <v>592</v>
+        <v>353</v>
+      </c>
+      <c r="K27" t="s">
+        <v>360</v>
       </c>
     </row>
     <row r="28" spans="1:16">
       <c r="A28" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B28" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C28" t="s">
         <v>160</v>
       </c>
       <c r="D28" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F28" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="G28">
         <v>2</v>
       </c>
       <c r="H28">
-        <v>40367001</v>
+        <v>40459001</v>
       </c>
       <c r="J28" s="6">
-        <v>472</v>
+        <v>368</v>
+      </c>
+      <c r="K28" t="s">
+        <v>360</v>
+      </c>
+      <c r="L28" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="29" spans="1:16">
       <c r="A29" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B29" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C29" t="s">
         <v>160</v>
       </c>
       <c r="D29" t="s">
-        <v>321</v>
+        <v>312</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
       <c r="F29" t="s">
-        <v>322</v>
+        <v>313</v>
       </c>
       <c r="G29">
         <v>2</v>
       </c>
       <c r="H29">
-        <v>40369001</v>
+        <v>40371001</v>
       </c>
       <c r="J29" s="6">
-        <v>320</v>
+        <v>592</v>
+      </c>
+      <c r="K29" t="s">
+        <v>360</v>
+      </c>
+      <c r="L29" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="30" spans="1:16">
       <c r="A30" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B30" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C30" t="s">
         <v>160</v>
       </c>
       <c r="D30" t="s">
-        <v>325</v>
+        <v>306</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>327</v>
+        <v>307</v>
       </c>
       <c r="F30" t="s">
-        <v>326</v>
+        <v>308</v>
       </c>
       <c r="G30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H30">
-        <v>40365001</v>
+        <v>40367001</v>
       </c>
       <c r="J30" s="6">
-        <v>303</v>
+        <v>472</v>
+      </c>
+      <c r="K30" t="s">
+        <v>360</v>
       </c>
     </row>
     <row r="31" spans="1:16">
       <c r="A31" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B31" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C31" t="s">
         <v>160</v>
       </c>
       <c r="D31" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="F31" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="G31">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H31">
-        <v>40365001</v>
+        <v>40369001</v>
       </c>
       <c r="J31" s="6">
-        <v>182</v>
+        <v>320</v>
+      </c>
+      <c r="K31" t="s">
+        <v>360</v>
       </c>
     </row>
     <row r="32" spans="1:16">
       <c r="A32" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B32" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C32" t="s">
         <v>160</v>
       </c>
       <c r="D32" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>316</v>
+        <v>325</v>
       </c>
       <c r="F32" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="G32">
         <v>1</v>
       </c>
       <c r="H32">
-        <v>40511001</v>
+        <v>40365001</v>
       </c>
       <c r="J32" s="6">
-        <v>168</v>
+        <v>303</v>
+      </c>
+      <c r="K32" t="s">
+        <v>360</v>
+      </c>
+      <c r="L32" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="33" spans="1:16">
       <c r="A33" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B33" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C33" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="D33" t="s">
-        <v>298</v>
+        <v>321</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="F33" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="G33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H33">
-        <v>40364001</v>
+        <v>40365001</v>
       </c>
       <c r="J33" s="6">
-        <v>202</v>
+        <v>179.21</v>
+      </c>
+      <c r="K33" t="s">
+        <v>0</v>
+      </c>
+      <c r="L33" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="34" spans="1:16">
       <c r="A34" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B34" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C34" t="s">
         <v>160</v>
       </c>
       <c r="D34" t="s">
+        <v>321</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="F34" t="s">
+        <v>322</v>
+      </c>
+      <c r="G34">
+        <v>1</v>
+      </c>
+      <c r="H34">
+        <v>40365001</v>
+      </c>
+      <c r="J34" s="6">
+        <v>182</v>
+      </c>
+      <c r="K34" t="s">
+        <v>360</v>
+      </c>
+      <c r="L34" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16">
+      <c r="A35" t="s">
         <v>298</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="B35" t="s">
+        <v>297</v>
+      </c>
+      <c r="C35" t="s">
+        <v>160</v>
+      </c>
+      <c r="D35" t="s">
+        <v>316</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="F35" t="s">
+        <v>317</v>
+      </c>
+      <c r="G35">
+        <v>1</v>
+      </c>
+      <c r="H35">
+        <v>40511001</v>
+      </c>
+      <c r="J35" s="6">
+        <v>168</v>
+      </c>
+      <c r="K35" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16">
+      <c r="A36" t="s">
+        <v>298</v>
+      </c>
+      <c r="B36" t="s">
+        <v>297</v>
+      </c>
+      <c r="C36" t="s">
+        <v>160</v>
+      </c>
+      <c r="D36" t="s">
         <v>296</v>
       </c>
-      <c r="F34" t="s">
-        <v>297</v>
-      </c>
-      <c r="G34">
+      <c r="E36" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="F36" t="s">
+        <v>315</v>
+      </c>
+      <c r="G36">
         <v>2</v>
       </c>
-      <c r="H34">
-        <v>40461001</v>
-      </c>
-      <c r="J34" s="6">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="35" spans="1:16">
-      <c r="D35" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="J35" s="6">
-        <f>SUM(J25:J34)</f>
-        <v>3114</v>
-      </c>
-      <c r="P35">
-        <f>J35</f>
-        <v>3114</v>
+      <c r="H36">
+        <v>40364001</v>
+      </c>
+      <c r="J36" s="6">
+        <v>202</v>
+      </c>
+      <c r="K36" t="s">
+        <v>360</v>
       </c>
     </row>
     <row r="37" spans="1:16">
       <c r="A37" t="s">
-        <v>234</v>
+        <v>298</v>
       </c>
       <c r="B37" t="s">
-        <v>171</v>
+        <v>297</v>
       </c>
       <c r="C37" t="s">
-        <v>238</v>
+        <v>160</v>
       </c>
       <c r="D37" t="s">
-        <v>239</v>
+        <v>296</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="G37" t="s">
-        <v>241</v>
-      </c>
-      <c r="J37">
-        <v>1099</v>
+        <v>294</v>
+      </c>
+      <c r="F37" t="s">
+        <v>295</v>
+      </c>
+      <c r="G37">
+        <v>2</v>
+      </c>
+      <c r="H37">
+        <v>40461001</v>
+      </c>
+      <c r="J37" s="6">
+        <v>154</v>
       </c>
       <c r="K37" t="s">
-        <v>242</v>
+        <v>360</v>
       </c>
     </row>
     <row r="38" spans="1:16">
-      <c r="A38" t="s">
-        <v>234</v>
-      </c>
-      <c r="B38" t="s">
-        <v>171</v>
-      </c>
-      <c r="C38" t="s">
-        <v>263</v>
-      </c>
-      <c r="D38" t="s">
-        <v>264</v>
-      </c>
-      <c r="E38" s="1"/>
-      <c r="G38">
-        <v>1</v>
-      </c>
-      <c r="J38">
-        <v>3500</v>
-      </c>
-      <c r="M38" s="4" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16">
-      <c r="A39" t="s">
-        <v>169</v>
-      </c>
-      <c r="B39" t="s">
-        <v>171</v>
-      </c>
-      <c r="C39" t="s">
-        <v>262</v>
-      </c>
-      <c r="D39" t="s">
-        <v>261</v>
-      </c>
-      <c r="E39" s="1"/>
-      <c r="G39">
-        <v>2</v>
-      </c>
-      <c r="J39">
-        <v>4000</v>
-      </c>
-      <c r="M39" s="4" t="s">
-        <v>254</v>
+      <c r="D38" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="J38" s="6">
+        <f>SUM(J27:J37)</f>
+        <v>3293.21</v>
+      </c>
+      <c r="P38">
+        <f>J38</f>
+        <v>3293.21</v>
       </c>
     </row>
     <row r="40" spans="1:16">
       <c r="A40" t="s">
-        <v>169</v>
+        <v>234</v>
       </c>
       <c r="B40" t="s">
         <v>171</v>
       </c>
       <c r="C40" t="s">
-        <v>263</v>
+        <v>238</v>
       </c>
       <c r="D40" t="s">
-        <v>264</v>
-      </c>
-      <c r="E40" s="1"/>
-      <c r="G40">
-        <v>1</v>
+        <v>239</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="G40" t="s">
+        <v>241</v>
       </c>
       <c r="J40">
-        <v>3500</v>
-      </c>
-      <c r="M40" s="4" t="s">
-        <v>254</v>
+        <v>1099</v>
+      </c>
+      <c r="K40" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="41" spans="1:16">
       <c r="A41" t="s">
-        <v>169</v>
+        <v>234</v>
       </c>
       <c r="B41" t="s">
         <v>171</v>
       </c>
       <c r="C41" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="D41" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="E41" s="1"/>
       <c r="G41">
         <v>1</v>
       </c>
       <c r="J41">
-        <v>3500</v>
-      </c>
-      <c r="M41" s="4" t="s">
+        <v>3555</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16">
+      <c r="A42" t="s">
+        <v>169</v>
+      </c>
+      <c r="B42" t="s">
+        <v>171</v>
+      </c>
+      <c r="C42" t="s">
+        <v>261</v>
+      </c>
+      <c r="D42" t="s">
+        <v>260</v>
+      </c>
+      <c r="E42" s="1"/>
+      <c r="G42">
+        <v>2</v>
+      </c>
+      <c r="J42">
+        <v>4000</v>
+      </c>
+      <c r="M42" s="4" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="42" spans="1:16">
-      <c r="D42" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="E42" s="1"/>
-      <c r="J42" s="6">
-        <f>SUM(J37:K41)</f>
-        <v>15599</v>
-      </c>
-      <c r="K42" t="s">
-        <v>260</v>
-      </c>
-      <c r="N42">
+    <row r="43" spans="1:16">
+      <c r="A43" t="s">
+        <v>169</v>
+      </c>
+      <c r="B43" t="s">
+        <v>171</v>
+      </c>
+      <c r="C43" t="s">
+        <v>262</v>
+      </c>
+      <c r="D43" t="s">
+        <v>263</v>
+      </c>
+      <c r="E43" s="1"/>
+      <c r="G43">
         <v>1</v>
       </c>
-      <c r="P42">
-        <f>J42</f>
-        <v>15599</v>
-      </c>
-    </row>
-    <row r="43" spans="1:16">
-      <c r="E43" s="1"/>
+      <c r="J43">
+        <v>4220</v>
+      </c>
     </row>
     <row r="44" spans="1:16">
       <c r="A44" t="s">
-        <v>135</v>
+        <v>169</v>
       </c>
       <c r="B44" t="s">
-        <v>243</v>
+        <v>171</v>
       </c>
       <c r="C44" t="s">
-        <v>244</v>
+        <v>264</v>
       </c>
       <c r="D44" t="s">
-        <v>245</v>
+        <v>265</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>246</v>
+        <v>366</v>
       </c>
       <c r="F44" t="s">
-        <v>247</v>
+        <v>365</v>
       </c>
       <c r="G44">
         <v>1</v>
       </c>
-      <c r="H44" t="s">
+      <c r="J44">
+        <v>4800</v>
+      </c>
+      <c r="M44" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16">
+      <c r="D45" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="E45" s="1"/>
+      <c r="J45" s="6">
+        <f>SUM(J40:K44)</f>
+        <v>17674</v>
+      </c>
+      <c r="K45" t="s">
+        <v>259</v>
+      </c>
+      <c r="N45">
+        <v>1</v>
+      </c>
+      <c r="P45">
+        <f>J45</f>
+        <v>17674</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16">
+      <c r="E46" s="1"/>
+    </row>
+    <row r="47" spans="1:16">
+      <c r="A47" t="s">
+        <v>135</v>
+      </c>
+      <c r="B47" t="s">
+        <v>243</v>
+      </c>
+      <c r="C47" t="s">
+        <v>244</v>
+      </c>
+      <c r="D47" t="s">
+        <v>245</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="F47" t="s">
+        <v>247</v>
+      </c>
+      <c r="G47">
+        <v>1</v>
+      </c>
+      <c r="H47" t="s">
         <v>137</v>
       </c>
-      <c r="J44">
+      <c r="J47">
         <v>900</v>
       </c>
-      <c r="K44" t="s">
+      <c r="K47" t="s">
         <v>248</v>
       </c>
-      <c r="L44" t="s">
+      <c r="L47" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="45" spans="1:16">
-      <c r="A45" t="s">
-        <v>149</v>
-      </c>
-      <c r="B45" t="s">
-        <v>136</v>
-      </c>
-      <c r="C45" t="s">
-        <v>251</v>
-      </c>
-      <c r="D45" t="s">
-        <v>252</v>
-      </c>
-      <c r="E45" s="1"/>
-      <c r="G45">
-        <v>2</v>
-      </c>
-      <c r="J45">
-        <v>3600</v>
-      </c>
-      <c r="K45" t="s">
-        <v>250</v>
-      </c>
-      <c r="L45" t="s">
-        <v>253</v>
-      </c>
-      <c r="M45" s="4" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="46" spans="1:16">
-      <c r="A46" t="s">
-        <v>255</v>
-      </c>
-      <c r="B46" t="s">
-        <v>136</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>256</v>
-      </c>
-      <c r="E46" s="1"/>
-      <c r="J46" s="6">
-        <f>SUM(J44:J45)</f>
-        <v>4500</v>
-      </c>
-      <c r="N46">
-        <v>1</v>
-      </c>
-      <c r="P46">
-        <f>J46</f>
-        <v>4500</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16">
-      <c r="E47" s="1"/>
     </row>
     <row r="48" spans="1:16">
       <c r="A48" t="s">
-        <v>167</v>
+        <v>149</v>
       </c>
       <c r="B48" t="s">
-        <v>278</v>
+        <v>136</v>
       </c>
       <c r="C48" t="s">
-        <v>225</v>
+        <v>251</v>
       </c>
       <c r="D48" t="s">
-        <v>224</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="F48" t="s">
-        <v>227</v>
-      </c>
+        <v>252</v>
+      </c>
+      <c r="E48" s="1"/>
       <c r="G48">
+        <v>2</v>
+      </c>
+      <c r="J48">
+        <v>3600</v>
+      </c>
+      <c r="K48" t="s">
+        <v>250</v>
+      </c>
+      <c r="L48" t="s">
+        <v>253</v>
+      </c>
+      <c r="M48" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16">
+      <c r="D49" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="E49" s="1"/>
+      <c r="J49" s="6">
+        <f>SUM(J47:J48)</f>
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16">
+      <c r="C50" t="s">
+        <v>353</v>
+      </c>
+      <c r="D50" t="s">
+        <v>355</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="F50" t="s">
+        <v>357</v>
+      </c>
+      <c r="G50">
         <v>1</v>
       </c>
-      <c r="J48">
-        <v>1273</v>
-      </c>
-      <c r="K48" t="s">
-        <v>138</v>
-      </c>
-      <c r="L48" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="49" spans="1:16">
-      <c r="A49" t="s">
-        <v>167</v>
-      </c>
-      <c r="B49" t="s">
-        <v>278</v>
-      </c>
-      <c r="D49" t="s">
-        <v>280</v>
-      </c>
-      <c r="E49" s="1"/>
-      <c r="J49">
-        <v>5000</v>
-      </c>
-      <c r="M49" s="4" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="50" spans="1:16">
-      <c r="A50" t="s">
-        <v>167</v>
-      </c>
-      <c r="B50" t="s">
-        <v>278</v>
-      </c>
-      <c r="D50" t="s">
-        <v>281</v>
-      </c>
-      <c r="E50" s="1"/>
-      <c r="J50">
-        <v>5000</v>
-      </c>
-      <c r="M50" s="4" t="s">
-        <v>254</v>
+      <c r="H50" t="s">
+        <v>356</v>
+      </c>
+      <c r="J50" s="8">
+        <v>2209</v>
+      </c>
+      <c r="K50" t="s">
+        <v>358</v>
+      </c>
+      <c r="L50" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="51" spans="1:16">
       <c r="A51" t="s">
-        <v>228</v>
+        <v>255</v>
       </c>
       <c r="B51" t="s">
-        <v>278</v>
-      </c>
-      <c r="C51" t="s">
-        <v>225</v>
-      </c>
-      <c r="D51" t="s">
-        <v>224</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>229</v>
-      </c>
-      <c r="F51" t="s">
-        <v>230</v>
-      </c>
-      <c r="G51">
+        <v>150</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="E51" s="1"/>
+      <c r="J51" s="6">
+        <f>SUM(J49:J50)</f>
+        <v>6709</v>
+      </c>
+      <c r="N51">
         <v>1</v>
       </c>
-      <c r="H51">
-        <v>185418</v>
-      </c>
-      <c r="J51">
-        <v>1107</v>
-      </c>
-      <c r="K51" t="s">
-        <v>138</v>
-      </c>
-      <c r="L51" t="s">
-        <v>148</v>
+      <c r="P51">
+        <f>J51</f>
+        <v>6709</v>
       </c>
     </row>
     <row r="52" spans="1:16">
-      <c r="A52" t="s">
-        <v>135</v>
-      </c>
-      <c r="B52" t="s">
-        <v>278</v>
-      </c>
-      <c r="D52" t="s">
-        <v>279</v>
-      </c>
       <c r="E52" s="1"/>
-      <c r="J52">
-        <v>5000</v>
-      </c>
-      <c r="M52" s="4" t="s">
-        <v>254</v>
-      </c>
     </row>
     <row r="53" spans="1:16">
       <c r="A53" t="s">
-        <v>135</v>
+        <v>167</v>
       </c>
       <c r="B53" t="s">
-        <v>142</v>
+        <v>276</v>
       </c>
       <c r="C53" t="s">
-        <v>139</v>
+        <v>225</v>
       </c>
       <c r="D53" t="s">
-        <v>143</v>
-      </c>
-      <c r="E53" t="s">
-        <v>144</v>
+        <v>224</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>226</v>
       </c>
       <c r="F53" t="s">
-        <v>145</v>
+        <v>227</v>
       </c>
       <c r="G53">
         <v>1</v>
       </c>
-      <c r="H53" t="s">
+      <c r="J53">
+        <v>1273</v>
+      </c>
+      <c r="K53" t="s">
+        <v>138</v>
+      </c>
+      <c r="L53" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16">
+      <c r="A54" t="s">
+        <v>167</v>
+      </c>
+      <c r="B54" t="s">
+        <v>276</v>
+      </c>
+      <c r="D54" t="s">
+        <v>278</v>
+      </c>
+      <c r="E54" s="1"/>
+      <c r="J54">
+        <v>5000</v>
+      </c>
+      <c r="M54" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16">
+      <c r="A55" t="s">
+        <v>167</v>
+      </c>
+      <c r="B55" t="s">
+        <v>276</v>
+      </c>
+      <c r="D55" t="s">
+        <v>279</v>
+      </c>
+      <c r="E55" s="1"/>
+      <c r="J55">
+        <v>5000</v>
+      </c>
+      <c r="M55" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16">
+      <c r="A56" t="s">
+        <v>228</v>
+      </c>
+      <c r="B56" t="s">
+        <v>276</v>
+      </c>
+      <c r="C56" t="s">
+        <v>225</v>
+      </c>
+      <c r="D56" t="s">
+        <v>224</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="F56" t="s">
+        <v>230</v>
+      </c>
+      <c r="G56">
+        <v>1</v>
+      </c>
+      <c r="H56">
+        <v>185418</v>
+      </c>
+      <c r="J56">
+        <v>1107</v>
+      </c>
+      <c r="K56" t="s">
+        <v>138</v>
+      </c>
+      <c r="L56" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16">
+      <c r="A57" t="s">
+        <v>157</v>
+      </c>
+      <c r="B57" t="s">
+        <v>276</v>
+      </c>
+      <c r="D57" t="s">
+        <v>364</v>
+      </c>
+      <c r="E57" s="1"/>
+      <c r="G57">
+        <v>1</v>
+      </c>
+      <c r="J57">
+        <v>2000</v>
+      </c>
+      <c r="M57" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16">
+      <c r="A58" t="s">
+        <v>135</v>
+      </c>
+      <c r="B58" t="s">
+        <v>276</v>
+      </c>
+      <c r="D58" t="s">
+        <v>277</v>
+      </c>
+      <c r="E58" s="1"/>
+      <c r="G58">
+        <v>1</v>
+      </c>
+      <c r="J58">
+        <v>5000</v>
+      </c>
+      <c r="M58" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16">
+      <c r="A59" t="s">
+        <v>135</v>
+      </c>
+      <c r="B59" t="s">
+        <v>276</v>
+      </c>
+      <c r="D59" t="s">
+        <v>364</v>
+      </c>
+      <c r="E59" s="1"/>
+      <c r="G59">
+        <v>1</v>
+      </c>
+      <c r="J59">
+        <v>2000</v>
+      </c>
+      <c r="M59" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16">
+      <c r="A60" t="s">
+        <v>135</v>
+      </c>
+      <c r="B60" t="s">
+        <v>142</v>
+      </c>
+      <c r="C60" t="s">
+        <v>139</v>
+      </c>
+      <c r="D60" t="s">
+        <v>143</v>
+      </c>
+      <c r="E60" t="s">
+        <v>144</v>
+      </c>
+      <c r="F60" t="s">
+        <v>145</v>
+      </c>
+      <c r="G60">
+        <v>1</v>
+      </c>
+      <c r="H60" t="s">
         <v>140</v>
       </c>
-      <c r="I53" t="s">
+      <c r="I60" t="s">
         <v>141</v>
       </c>
-      <c r="J53">
+      <c r="J60">
         <v>1818</v>
       </c>
-      <c r="K53" t="s">
+      <c r="K60" t="s">
         <v>146</v>
       </c>
-      <c r="L53" t="s">
+      <c r="L60" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="54" spans="1:16">
-      <c r="D54" s="7" t="s">
-        <v>276</v>
-      </c>
-      <c r="J54">
-        <f>SUM(J48:J53)</f>
-        <v>19198</v>
-      </c>
-      <c r="L54" t="s">
-        <v>257</v>
-      </c>
-      <c r="N54">
+    <row r="61" spans="1:16">
+      <c r="D61" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="J61">
+        <f>SUM(J53:J60)</f>
+        <v>23198</v>
+      </c>
+      <c r="L61" t="s">
+        <v>256</v>
+      </c>
+      <c r="N61">
         <v>2</v>
       </c>
     </row>
-    <row r="55" spans="1:16">
-      <c r="D55" s="3" t="s">
-        <v>277</v>
-      </c>
-      <c r="J55">
-        <f>SUM(J48:J53)</f>
-        <v>19198</v>
-      </c>
-      <c r="N55">
+    <row r="62" spans="1:16">
+      <c r="D62" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="J62">
+        <f>SUM(J53:J60)</f>
+        <v>23198</v>
+      </c>
+      <c r="N62">
         <v>1</v>
       </c>
-      <c r="P55">
-        <f>J55</f>
-        <v>19198</v>
-      </c>
-    </row>
-    <row r="57" spans="1:16">
-      <c r="B57" t="s">
+      <c r="P62">
+        <f>J62</f>
+        <v>23198</v>
+      </c>
+    </row>
+    <row r="64" spans="1:16">
+      <c r="A64" t="s">
+        <v>135</v>
+      </c>
+      <c r="B64" t="s">
+        <v>368</v>
+      </c>
+      <c r="C64" t="s">
+        <v>369</v>
+      </c>
+      <c r="D64" t="s">
+        <v>370</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="F64" t="s">
+        <v>372</v>
+      </c>
+      <c r="G64">
+        <v>1</v>
+      </c>
+      <c r="H64">
+        <v>514708</v>
+      </c>
+      <c r="J64">
+        <v>3682</v>
+      </c>
+      <c r="K64" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="65" spans="1:16">
+      <c r="A65" t="s">
+        <v>135</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="P65">
+        <f>SUM(J64:J64)</f>
+        <v>3682</v>
+      </c>
+    </row>
+    <row r="67" spans="1:16">
+      <c r="B67" t="s">
+        <v>286</v>
+      </c>
+      <c r="J67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:16">
+      <c r="B68" t="s">
+        <v>287</v>
+      </c>
+      <c r="J68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:16">
+      <c r="B69" t="s">
         <v>288</v>
       </c>
-      <c r="J57">
-        <v>47000</v>
-      </c>
-    </row>
-    <row r="58" spans="1:16">
-      <c r="B58" t="s">
-        <v>289</v>
-      </c>
-      <c r="J58">
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="59" spans="1:16">
-      <c r="B59" t="s">
-        <v>290</v>
-      </c>
-      <c r="J59">
-        <v>14000</v>
-      </c>
-    </row>
-    <row r="60" spans="1:16">
-      <c r="D60" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="J60" s="6">
-        <f>SUM(J57:J59)</f>
-        <v>91000</v>
-      </c>
-      <c r="L60" t="s">
-        <v>283</v>
-      </c>
-      <c r="O60">
-        <v>0.9</v>
-      </c>
-      <c r="P60">
-        <f>J60*O60</f>
-        <v>81900</v>
-      </c>
-    </row>
-    <row r="65" spans="1:16">
-      <c r="B65" t="s">
+      <c r="J69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:16">
+      <c r="D70" t="s">
+        <v>361</v>
+      </c>
+      <c r="J70">
+        <v>83000</v>
+      </c>
+    </row>
+    <row r="71" spans="1:16">
+      <c r="D71" t="s">
+        <v>362</v>
+      </c>
+      <c r="G71">
+        <v>1</v>
+      </c>
+      <c r="J71">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="72" spans="1:16">
+      <c r="D72" t="s">
+        <v>363</v>
+      </c>
+      <c r="G72">
+        <v>2</v>
+      </c>
+      <c r="J72">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="73" spans="1:16">
+      <c r="D73" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="J73" s="6">
+        <f>SUM(J67:J72)</f>
+        <v>84197</v>
+      </c>
+      <c r="L73" t="s">
+        <v>281</v>
+      </c>
+      <c r="O73">
+        <v>1</v>
+      </c>
+      <c r="P73">
+        <f>J73*O73</f>
+        <v>84197</v>
+      </c>
+    </row>
+    <row r="78" spans="1:16">
+      <c r="B78" t="s">
+        <v>266</v>
+      </c>
+      <c r="C78" t="s">
         <v>267</v>
       </c>
-      <c r="C65" t="s">
+      <c r="D78" t="s">
         <v>269</v>
       </c>
-      <c r="D65" t="s">
+      <c r="J78">
+        <v>44000</v>
+      </c>
+      <c r="K78" t="s">
+        <v>332</v>
+      </c>
+      <c r="L78" t="s">
+        <v>333</v>
+      </c>
+      <c r="M78" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="79" spans="1:16">
+      <c r="A79" t="s">
+        <v>169</v>
+      </c>
+      <c r="B79" t="s">
+        <v>266</v>
+      </c>
+      <c r="D79" t="s">
+        <v>331</v>
+      </c>
+      <c r="J79">
+        <v>4000</v>
+      </c>
+      <c r="M79" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="80" spans="1:16">
+      <c r="A80" t="s">
+        <v>167</v>
+      </c>
+      <c r="B80" t="s">
+        <v>266</v>
+      </c>
+      <c r="D80" t="s">
+        <v>330</v>
+      </c>
+      <c r="J80">
+        <v>4000</v>
+      </c>
+      <c r="M80" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="81" spans="1:16">
+      <c r="A81" t="s">
+        <v>326</v>
+      </c>
+      <c r="B81" t="s">
+        <v>266</v>
+      </c>
+      <c r="D81" t="s">
+        <v>327</v>
+      </c>
+      <c r="J81">
+        <v>3500</v>
+      </c>
+      <c r="M81" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="82" spans="1:16">
+      <c r="A82" t="s">
+        <v>328</v>
+      </c>
+      <c r="B82" t="s">
+        <v>266</v>
+      </c>
+      <c r="D82" t="s">
+        <v>329</v>
+      </c>
+      <c r="J82">
+        <v>6000</v>
+      </c>
+      <c r="M82" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="83" spans="1:16">
+      <c r="A83" t="s">
+        <v>268</v>
+      </c>
+      <c r="B83" t="s">
+        <v>266</v>
+      </c>
+      <c r="D83" t="s">
+        <v>270</v>
+      </c>
+      <c r="J83">
+        <v>2000</v>
+      </c>
+      <c r="M83" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="84" spans="1:16">
+      <c r="B84" t="s">
+        <v>266</v>
+      </c>
+      <c r="D84" t="s">
         <v>271</v>
       </c>
-      <c r="J65">
-        <v>44000</v>
-      </c>
-      <c r="K65" t="s">
-        <v>268</v>
-      </c>
-      <c r="M65" s="4" t="s">
+      <c r="J84">
+        <v>4500</v>
+      </c>
+      <c r="M84" s="4" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="66" spans="1:16">
-      <c r="A66" t="s">
-        <v>169</v>
-      </c>
-      <c r="B66" t="s">
-        <v>267</v>
-      </c>
-      <c r="D66" t="s">
-        <v>333</v>
-      </c>
-      <c r="J66">
-        <v>4000</v>
-      </c>
-      <c r="M66" s="4" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="67" spans="1:16">
-      <c r="A67" t="s">
-        <v>167</v>
-      </c>
-      <c r="B67" t="s">
-        <v>267</v>
-      </c>
-      <c r="D67" t="s">
-        <v>332</v>
-      </c>
-      <c r="J67">
-        <v>4000</v>
-      </c>
-      <c r="M67" s="4" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="68" spans="1:16">
-      <c r="A68" t="s">
-        <v>328</v>
-      </c>
-      <c r="B68" t="s">
-        <v>267</v>
-      </c>
-      <c r="D68" t="s">
-        <v>329</v>
-      </c>
-      <c r="J68">
-        <v>3500</v>
-      </c>
-      <c r="M68" s="4" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="69" spans="1:16">
-      <c r="A69" t="s">
-        <v>330</v>
-      </c>
-      <c r="B69" t="s">
-        <v>267</v>
-      </c>
-      <c r="D69" t="s">
-        <v>331</v>
-      </c>
-      <c r="J69">
-        <v>6000</v>
-      </c>
-      <c r="M69" s="4" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="70" spans="1:16">
-      <c r="A70" t="s">
-        <v>270</v>
-      </c>
-      <c r="B70" t="s">
-        <v>267</v>
-      </c>
-      <c r="D70" t="s">
+    <row r="85" spans="1:16">
+      <c r="D85" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="J70">
-        <v>2000</v>
-      </c>
-      <c r="M70" s="4" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="71" spans="1:16">
-      <c r="B71" t="s">
-        <v>267</v>
-      </c>
-      <c r="D71" t="s">
-        <v>273</v>
-      </c>
-      <c r="J71">
-        <v>4500</v>
-      </c>
-      <c r="M71" s="4" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="72" spans="1:16">
-      <c r="D72" s="3" t="s">
-        <v>274</v>
-      </c>
-      <c r="J72" s="6">
-        <f>SUM(J65:J71)</f>
+      <c r="J85" s="6">
+        <f>SUM(J78:J84)</f>
         <v>68000</v>
-      </c>
-      <c r="N72">
-        <v>1</v>
-      </c>
-      <c r="P72">
-        <f>J72</f>
-        <v>68000</v>
-      </c>
-    </row>
-    <row r="74" spans="1:16">
-      <c r="D74" s="7" t="s">
-        <v>294</v>
-      </c>
-      <c r="J74">
-        <v>30000</v>
-      </c>
-      <c r="M74" s="4" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="75" spans="1:16">
-      <c r="D75" s="7" t="s">
-        <v>293</v>
-      </c>
-      <c r="J75">
-        <v>20000</v>
-      </c>
-      <c r="M75" s="4" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="76" spans="1:16">
-      <c r="D76" s="7" t="s">
-        <v>292</v>
-      </c>
-      <c r="J76">
-        <v>40000</v>
-      </c>
-      <c r="M76" s="4" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="77" spans="1:16">
-      <c r="D77" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="J77" s="6">
-        <f>SUM(J74:J76)</f>
-        <v>90000</v>
-      </c>
-      <c r="N77">
-        <v>1</v>
-      </c>
-      <c r="P77">
-        <f>J77</f>
-        <v>90000</v>
-      </c>
-    </row>
-    <row r="79" spans="1:16">
-      <c r="J79">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" spans="1:16">
-      <c r="J80">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" spans="4:16">
-      <c r="D81" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="J81" s="6">
-        <f>SUM(J79:J80)</f>
-        <v>0</v>
-      </c>
-      <c r="N81">
-        <v>1</v>
-      </c>
-      <c r="P81">
-        <f>J81</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" spans="4:16">
-      <c r="J83">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="84" spans="4:16">
-      <c r="J84">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="85" spans="4:16">
-      <c r="D85" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="J85" s="6">
-        <f>SUM(J83:J84)</f>
-        <v>0</v>
       </c>
       <c r="N85">
         <v>1</v>
       </c>
       <c r="P85">
         <f>J85</f>
+        <v>68000</v>
+      </c>
+    </row>
+    <row r="87" spans="1:16">
+      <c r="D87" s="7" t="s">
+        <v>292</v>
+      </c>
+      <c r="J87">
+        <v>60000</v>
+      </c>
+      <c r="M87" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="88" spans="1:16">
+      <c r="D88" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="J88">
+        <v>20000</v>
+      </c>
+      <c r="M88" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="89" spans="1:16">
+      <c r="D89" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="J89">
+        <v>20000</v>
+      </c>
+      <c r="M89" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="90" spans="1:16">
+      <c r="D90" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="J90" s="6">
+        <f>SUM(J87:J89)</f>
+        <v>100000</v>
+      </c>
+      <c r="N90">
+        <v>1</v>
+      </c>
+      <c r="P90">
+        <f>J90</f>
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="92" spans="1:16">
+      <c r="B92" t="s">
+        <v>339</v>
+      </c>
+      <c r="D92" t="s">
+        <v>340</v>
+      </c>
+      <c r="J92">
+        <v>9200</v>
+      </c>
+      <c r="K92" t="s">
+        <v>341</v>
+      </c>
+      <c r="L92" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="93" spans="1:16">
+      <c r="J93">
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="4:16">
-      <c r="D87" s="5" t="s">
-        <v>258</v>
-      </c>
-      <c r="J87" s="2"/>
-      <c r="N87">
+    <row r="94" spans="1:16">
+      <c r="D94" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="J94" s="6">
+        <f>SUM(J92:J93)</f>
+        <v>9200</v>
+      </c>
+      <c r="N94">
+        <v>1</v>
+      </c>
+      <c r="P94">
+        <f>J94</f>
+        <v>9200</v>
+      </c>
+    </row>
+    <row r="96" spans="1:16">
+      <c r="J96">
         <v>0</v>
       </c>
-      <c r="P87" s="2">
-        <f>SUM(P1:P76)</f>
-        <v>205390.97</v>
+    </row>
+    <row r="97" spans="2:16">
+      <c r="J97">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="2:16">
+      <c r="D98" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="J98" s="6">
+        <f>SUM(J96:J97)</f>
+        <v>0</v>
+      </c>
+      <c r="N98">
+        <v>1</v>
+      </c>
+      <c r="P98">
+        <f>J98</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="2:16">
+      <c r="B100" t="s">
+        <v>345</v>
+      </c>
+      <c r="D100" t="s">
+        <v>344</v>
+      </c>
+      <c r="J100">
+        <v>138000</v>
+      </c>
+    </row>
+    <row r="101" spans="2:16">
+      <c r="B101" t="s">
+        <v>347</v>
+      </c>
+      <c r="D101" t="s">
+        <v>346</v>
+      </c>
+      <c r="J101">
+        <v>1500</v>
+      </c>
+      <c r="L101" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="102" spans="2:16">
+      <c r="B102" t="s">
+        <v>347</v>
+      </c>
+      <c r="D102" t="s">
+        <v>349</v>
+      </c>
+      <c r="J102">
+        <v>2000</v>
+      </c>
+      <c r="L102" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="103" spans="2:16">
+      <c r="D103" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="J103" s="6">
+        <f>SUM(J100:J102)</f>
+        <v>141500</v>
+      </c>
+      <c r="N103">
+        <v>1</v>
+      </c>
+      <c r="P103">
+        <f>J103</f>
+        <v>141500</v>
+      </c>
+    </row>
+    <row r="107" spans="2:16">
+      <c r="D107" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="J107" s="2"/>
+      <c r="N107">
+        <v>0</v>
+      </c>
+      <c r="P107" s="2">
+        <f>SUM(P1:P106)</f>
+        <v>476247.18</v>
       </c>
     </row>
   </sheetData>
@@ -3691,34 +4322,40 @@
     <hyperlink ref="E6" r:id="rId1"/>
     <hyperlink ref="E5" r:id="rId2"/>
     <hyperlink ref="E4" r:id="rId3"/>
-    <hyperlink ref="E10" r:id="rId4"/>
+    <hyperlink ref="E11" r:id="rId4"/>
     <hyperlink ref="E3" r:id="rId5"/>
-    <hyperlink ref="E11" r:id="rId6"/>
-    <hyperlink ref="E12" r:id="rId7"/>
+    <hyperlink ref="E12" r:id="rId6"/>
+    <hyperlink ref="E13" r:id="rId7"/>
     <hyperlink ref="E7" r:id="rId8"/>
     <hyperlink ref="E8" r:id="rId9"/>
-    <hyperlink ref="E13" r:id="rId10"/>
-    <hyperlink ref="E14" r:id="rId11"/>
-    <hyperlink ref="E15" r:id="rId12"/>
-    <hyperlink ref="E16" r:id="rId13"/>
-    <hyperlink ref="E17" r:id="rId14"/>
-    <hyperlink ref="E18" r:id="rId15"/>
-    <hyperlink ref="E51" r:id="rId16"/>
-    <hyperlink ref="E48" r:id="rId17"/>
-    <hyperlink ref="E19" r:id="rId18"/>
-    <hyperlink ref="E20" r:id="rId19"/>
-    <hyperlink ref="E37" r:id="rId20"/>
-    <hyperlink ref="E34" r:id="rId21" display="2 of GROHE Bau Cosmopolitan | Badaccessoires - Handtuch | Bademantelhaken | 40461001"/>
-    <hyperlink ref="E9" r:id="rId22"/>
-    <hyperlink ref="E25" r:id="rId23"/>
-    <hyperlink ref="E28" r:id="rId24"/>
-    <hyperlink ref="E26" r:id="rId25"/>
-    <hyperlink ref="E27" r:id="rId26"/>
-    <hyperlink ref="E33" r:id="rId27"/>
-    <hyperlink ref="E32" r:id="rId28"/>
-    <hyperlink ref="E29" r:id="rId29" display="2 of Grohe Essentials Halter, Glas Seifenschale, chrom, 40369001"/>
-    <hyperlink ref="E31" r:id="rId30"/>
-    <hyperlink ref="E30" r:id="rId31"/>
+    <hyperlink ref="E14" r:id="rId10"/>
+    <hyperlink ref="E15" r:id="rId11"/>
+    <hyperlink ref="E16" r:id="rId12"/>
+    <hyperlink ref="E17" r:id="rId13"/>
+    <hyperlink ref="E18" r:id="rId14"/>
+    <hyperlink ref="E19" r:id="rId15"/>
+    <hyperlink ref="E56" r:id="rId16"/>
+    <hyperlink ref="E53" r:id="rId17"/>
+    <hyperlink ref="E21" r:id="rId18"/>
+    <hyperlink ref="E22" r:id="rId19"/>
+    <hyperlink ref="E40" r:id="rId20"/>
+    <hyperlink ref="E37" r:id="rId21" display="2 of GROHE Bau Cosmopolitan | Badaccessoires - Handtuch | Bademantelhaken | 40461001"/>
+    <hyperlink ref="E10" r:id="rId22"/>
+    <hyperlink ref="E27" r:id="rId23"/>
+    <hyperlink ref="E30" r:id="rId24"/>
+    <hyperlink ref="E28" r:id="rId25"/>
+    <hyperlink ref="E29" r:id="rId26"/>
+    <hyperlink ref="E36" r:id="rId27"/>
+    <hyperlink ref="E35" r:id="rId28"/>
+    <hyperlink ref="E31" r:id="rId29" display="2 of Grohe Essentials Halter, Glas Seifenschale, chrom, 40369001"/>
+    <hyperlink ref="E34" r:id="rId30"/>
+    <hyperlink ref="E32" r:id="rId31"/>
+    <hyperlink ref="E50" r:id="rId32"/>
+    <hyperlink ref="E33" r:id="rId33"/>
+    <hyperlink ref="E44" r:id="rId34"/>
+    <hyperlink ref="E64" r:id="rId35"/>
+    <hyperlink ref="E20" r:id="rId36"/>
+    <hyperlink ref="E9" r:id="rId37"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
@@ -4125,7 +4762,7 @@
         <v>28</v>
       </c>
       <c r="E35">
-        <f>G35*H35</f>
+        <f t="shared" ref="E35:E41" si="0">G35*H35</f>
         <v>2000</v>
       </c>
       <c r="F35">
@@ -4149,7 +4786,7 @@
         <v>29</v>
       </c>
       <c r="E36">
-        <f>G36*H36</f>
+        <f t="shared" si="0"/>
         <v>144</v>
       </c>
       <c r="F36" t="s">
@@ -4173,7 +4810,7 @@
         <v>32</v>
       </c>
       <c r="E37">
-        <f>G37*H37</f>
+        <f t="shared" si="0"/>
         <v>120</v>
       </c>
       <c r="F37" t="s">
@@ -4197,7 +4834,7 @@
         <v>31</v>
       </c>
       <c r="E38">
-        <f>G38*H38</f>
+        <f t="shared" si="0"/>
         <v>240</v>
       </c>
       <c r="F38">
@@ -4221,7 +4858,7 @@
         <v>33</v>
       </c>
       <c r="E39">
-        <f>G39*H39</f>
+        <f t="shared" si="0"/>
         <v>624</v>
       </c>
       <c r="F39" t="s">
@@ -4245,7 +4882,7 @@
         <v>37</v>
       </c>
       <c r="E40">
-        <f>G40*H40</f>
+        <f t="shared" si="0"/>
         <v>291.2</v>
       </c>
       <c r="F40" t="s">
@@ -4269,7 +4906,7 @@
         <v>38</v>
       </c>
       <c r="E41">
-        <f>G41*H41</f>
+        <f t="shared" si="0"/>
         <v>665.6</v>
       </c>
       <c r="F41" t="s">

</xml_diff>